<commit_message>
Update osmolality chart labels and Y-axis ticks
Use 25-unit Y-axis divisions, rename Sample to Lote and Specification
range to Rango de aceptación, and remove the DO8 annotation.

Co-authored-by: Smansilla98 <Smansilla98@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/osmolality_results/osmolality_results.xlsx
+++ b/osmolality_results/osmolality_results.xlsx
@@ -249,7 +249,7 @@
           <idx val="1"/>
           <order val="1"/>
           <tx>
-            <v>Specification range</v>
+            <v>Rango de aceptación</v>
           </tx>
           <spPr>
             <a:solidFill>
@@ -283,7 +283,7 @@
           <idx val="2"/>
           <order val="2"/>
           <tx>
-            <v>Sample 1</v>
+            <v>Lote 1</v>
           </tx>
           <spPr>
             <a:ln>
@@ -321,7 +321,7 @@
           <idx val="3"/>
           <order val="3"/>
           <tx>
-            <v>Sample 2</v>
+            <v>Lote 2</v>
           </tx>
           <spPr>
             <a:ln>
@@ -411,6 +411,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <majorUnit val="25"/>
       </valAx>
       <valAx>
         <axId val="20"/>
@@ -880,22 +881,22 @@
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Sample 1 (mOsm/kg)</t>
+          <t>Lote 1 (mOsm/kg)</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Sample 2 (mOsm/kg)</t>
+          <t>Lote 2 (mOsm/kg)</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Sample 1 Status</t>
+          <t>Lote 1 Status</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Sample 2 Status</t>
+          <t>Lote 2 Status</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
@@ -915,12 +916,12 @@
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
-          <t>Sample 1 Y</t>
+          <t>Lote 1 Y</t>
         </is>
       </c>
       <c r="L1" s="3" t="inlineStr">
         <is>
-          <t>Sample 2 Y</t>
+          <t>Lote 2 Y</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1298,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Units: mOsm/kg. Markers: Sample 1 (orange), Sample 2 (green).</t>
+          <t>Units: mOsm/kg. Markers: Lote 1 (orange), Lote 2 (green).</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1334,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>X axis: products (DO1–DO8) | Y axis: osmolality (mOsm/kg) | Shade: specification range | Circles: Sample 1 &amp; Sample 2</t>
+          <t>X axis: products (DO1–DO8) | Y axis: osmolality (mOsm/kg), step 25 | Shade: Rango de aceptación | Circles: Lote 1 &amp; Lote 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Translate chart axis labels to Spanish
Rename Y axis to Osmolalidad (mOsm/kg) and X axis to Producto.

Co-authored-by: Smansilla98 <Smansilla98@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/osmolality_results/osmolality_results.xlsx
+++ b/osmolality_results/osmolality_results.xlsx
@@ -373,7 +373,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Product</a:t>
+                  <a:t>Producto</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -402,7 +402,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Osmolality (mOsm/kg)</a:t>
+                  <a:t>Osmolalidad (mOsm/kg)</a:t>
                 </a:r>
               </a:p>
             </rich>

</xml_diff>

<commit_message>
Add bold laboratory labels under DO chart X-axis
Map DO1–DO8 to laboratories B/E/F/G/H/I/J with G spanning DO4–DO5,
and rename the axis title to Laboratorio/Producto.

Co-authored-by: Smansilla98 <Smansilla98@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/osmolality_results/osmolality_results.xlsx
+++ b/osmolality_results/osmolality_results.xlsx
@@ -241,7 +241,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$H$2:$H$9</f>
+              <f>'Data'!$I$2:$I$9</f>
             </numRef>
           </val>
         </ser>
@@ -269,7 +269,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$I$2:$I$9</f>
+              <f>'Data'!$J$2:$J$9</f>
             </numRef>
           </val>
         </ser>
@@ -308,12 +308,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'Data'!$J$2:$J$9</f>
+              <f>'Data'!$K$2:$K$9</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'Data'!$K$2:$K$9</f>
+              <f>'Data'!$L$2:$L$9</f>
             </numRef>
           </yVal>
         </ser>
@@ -346,12 +346,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'Data'!$J$2:$J$9</f>
+              <f>'Data'!$K$2:$K$9</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'Data'!$L$2:$L$9</f>
+              <f>'Data'!$M$2:$M$9</f>
             </numRef>
           </yVal>
         </ser>
@@ -373,7 +373,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Producto</a:t>
+                  <a:t>Laboratorio/Producto</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -846,21 +846,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col hidden="1" width="14" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col hidden="1" width="14" customWidth="1" min="9" max="9"/>
-    <col hidden="1" width="10" customWidth="1" min="10" max="10"/>
-    <col hidden="1" width="12" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="14" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="10" customWidth="1" min="11" max="11"/>
     <col hidden="1" width="12" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -871,55 +872,60 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
+          <t>Laboratorio</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
           <t>Spec Min (mOsm/kg)</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Spec Max (mOsm/kg)</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Lote 1 (mOsm/kg)</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Lote 2 (mOsm/kg)</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Lote 1 Status</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Lote 2 Status</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Base (hidden)</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Range Height</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>X Index</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Lote 1 Y</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Lote 2 Y</t>
         </is>
@@ -931,41 +937,46 @@
           <t>DO1</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio B</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>320</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="E2" s="4" t="n">
         <v>282</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="F2" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="I2" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="J2" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="K2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>282</v>
       </c>
-      <c r="L2" s="4" t="n">
+      <c r="M2" s="4" t="n">
         <v>280</v>
       </c>
     </row>
@@ -975,41 +986,46 @@
           <t>DO2</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio E</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>240</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>340</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="E3" s="4" t="n">
         <v>286</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="F3" s="4" t="n">
         <v>283</v>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="I3" s="4" t="n">
         <v>240</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="J3" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="K3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="L3" s="4" t="n">
         <v>286</v>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="M3" s="4" t="n">
         <v>283</v>
       </c>
     </row>
@@ -1019,41 +1035,46 @@
           <t>DO3</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio F</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>250</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>350</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="E4" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="F4" s="4" t="n">
         <v>281</v>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="I4" s="4" t="n">
         <v>250</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="L4" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="M4" s="4" t="n">
         <v>281</v>
       </c>
     </row>
@@ -1063,41 +1084,46 @@
           <t>DO4</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio G</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>260</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>320</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="E5" s="4" t="n">
         <v>281</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>276</v>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="I5" s="4" t="n">
         <v>260</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="J5" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="K5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="L5" s="4" t="n">
         <v>281</v>
       </c>
-      <c r="L5" s="4" t="n">
+      <c r="M5" s="4" t="n">
         <v>276</v>
       </c>
     </row>
@@ -1107,41 +1133,46 @@
           <t>DO5</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio G</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>260</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>320</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="E6" s="4" t="n">
         <v>276</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="F6" s="4" t="n">
         <v>275</v>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="I6" s="4" t="n">
         <v>260</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="J6" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="K6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="L6" s="4" t="n">
         <v>276</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="M6" s="4" t="n">
         <v>275</v>
       </c>
     </row>
@@ -1151,41 +1182,46 @@
           <t>DO6</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio H</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>240</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>370</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="E7" s="4" t="n">
         <v>287</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="F7" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="I7" s="4" t="n">
         <v>240</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="J7" s="4" t="n">
         <v>130</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="K7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="K7" s="4" t="n">
+      <c r="L7" s="4" t="n">
         <v>287</v>
       </c>
-      <c r="L7" s="4" t="n">
+      <c r="M7" s="4" t="n">
         <v>280</v>
       </c>
     </row>
@@ -1195,41 +1231,46 @@
           <t>DO7</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio I</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
         <v>270</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="D8" s="4" t="n">
         <v>330</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="E8" s="4" t="n">
         <v>310</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="F8" s="4" t="n">
         <v>312</v>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="I8" s="4" t="n">
         <v>270</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="J8" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="K8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="L8" s="4" t="n">
         <v>310</v>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="M8" s="4" t="n">
         <v>312</v>
       </c>
     </row>
@@ -1241,43 +1282,48 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
+          <t>Laboratorio J</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="E9" s="4" t="n">
         <v>573</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="F9" s="4" t="n">
         <v>579</v>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>N/A (no specification)</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>N/A (no specification)</t>
         </is>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="I9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="K9" s="4" t="n">
+      <c r="L9" s="4" t="n">
         <v>573</v>
       </c>
-      <c r="L9" s="4" t="n">
+      <c r="M9" s="4" t="n">
         <v>579</v>
       </c>
     </row>
@@ -1291,7 +1337,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Specification range is shown as a shaded band for each product. DO8 has no specification; only sample markers are displayed.</t>
+          <t>Rango de aceptación shown as a shaded band. DO8 has no specification; only lote markers are displayed. X-axis shows product and belonging Laboratorio.</t>
         </is>
       </c>
     </row>
@@ -1304,8 +1350,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A13:H13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1334,7 +1380,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>X axis: products (DO1–DO8) | Y axis: osmolality (mOsm/kg), step 25 | Shade: Rango de aceptación | Circles: Lote 1 &amp; Lote 2</t>
+          <t>Eje X: Producto (DO1–DO8) + Laboratorio | Eje Y: Osmolalidad (mOsm/kg), paso 25 | Sombra: Rango de aceptación | Círculos: Lote 1 &amp; Lote 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add DO9 and asterisk markers to DO osmolality chart
Include Laboratorio K for DO9 with asterisk at 288, and mark DO8 with
an asterisk at 574 while keeping existing lote markers.

Co-authored-by: Smansilla98 <Smansilla98@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/osmolality_results/osmolality_results.xlsx
+++ b/osmolality_results/osmolality_results.xlsx
@@ -236,12 +236,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Data'!$A$2:$A$9</f>
+              <f>'Data'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$I$2:$I$9</f>
+              <f>'Data'!$J$2:$J$10</f>
             </numRef>
           </val>
         </ser>
@@ -264,12 +264,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Data'!$A$2:$A$9</f>
+              <f>'Data'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$J$2:$J$9</f>
+              <f>'Data'!$K$2:$K$10</f>
             </numRef>
           </val>
         </ser>
@@ -308,12 +308,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'Data'!$K$2:$K$9</f>
+              <f>'Data'!$L$2:$L$10</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'Data'!$L$2:$L$9</f>
+              <f>'Data'!$M$2:$M$10</f>
             </numRef>
           </yVal>
         </ser>
@@ -346,12 +346,50 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'Data'!$K$2:$K$9</f>
+              <f>'Data'!$L$2:$L$10</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'Data'!$M$2:$M$9</f>
+              <f>'Data'!$N$2:$N$10</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <v>*</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="star"/>
+            <size val="10"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'Data'!$L$2:$L$10</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Data'!$O$2:$O$10</f>
             </numRef>
           </yVal>
         </ser>
@@ -440,10 +478,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>15</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6480000" cy="4320000"/>
+    <ext cx="7200000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -470,7 +508,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9144000" cy="5334000"/>
+    <ext cx="9715500" cy="5524500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -783,7 +821,7 @@
   <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="90" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -796,14 +834,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>All products with a specification range are within limits for both samples.</t>
+          <t>All products with a specification range are within limits for both lots.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DO8 has no specification range; measured values are ~573–579 mOsm/kg.</t>
+          <t>DO8 has no specification (lotes ~573–579; asterisk at 574). DO9 (Laboratorio K) has asterisk-only value at 288 mOsm/kg.</t>
         </is>
       </c>
     </row>
@@ -846,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -855,13 +893,15 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col hidden="1" width="14" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
     <col hidden="1" width="14" customWidth="1" min="10" max="10"/>
-    <col hidden="1" width="10" customWidth="1" min="11" max="11"/>
-    <col hidden="1" width="12" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="14" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="10" customWidth="1" min="12" max="12"/>
     <col hidden="1" width="12" customWidth="1" min="13" max="13"/>
+    <col hidden="1" width="12" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -897,37 +937,47 @@
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
+          <t>Asterisk (mOsm/kg)</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
           <t>Lote 1 Status</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Lote 2 Status</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Base (hidden)</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Range Height</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>X Index</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Lote 1 Y</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Lote 2 Y</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>Asterisk Y</t>
         </is>
       </c>
     </row>
@@ -954,31 +1004,37 @@
       <c r="F2" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="J2" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="K2" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L2" s="4" t="n">
+      <c r="M2" s="4" t="n">
         <v>282</v>
       </c>
-      <c r="M2" s="4" t="n">
+      <c r="N2" s="4" t="n">
         <v>280</v>
       </c>
+      <c r="O2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1003,31 +1059,37 @@
       <c r="F3" s="4" t="n">
         <v>283</v>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="J3" s="4" t="n">
         <v>240</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="K3" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="L3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="M3" s="4" t="n">
         <v>286</v>
       </c>
-      <c r="M3" s="4" t="n">
+      <c r="N3" s="4" t="n">
         <v>283</v>
       </c>
+      <c r="O3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1052,31 +1114,37 @@
       <c r="F4" s="4" t="n">
         <v>281</v>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>250</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="L4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="M4" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="N4" s="4" t="n">
         <v>281</v>
       </c>
+      <c r="O4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1101,31 +1169,37 @@
       <c r="F5" s="4" t="n">
         <v>276</v>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="J5" s="4" t="n">
         <v>260</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="K5" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="L5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="L5" s="4" t="n">
+      <c r="M5" s="4" t="n">
         <v>281</v>
       </c>
-      <c r="M5" s="4" t="n">
+      <c r="N5" s="4" t="n">
         <v>276</v>
       </c>
+      <c r="O5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1150,31 +1224,37 @@
       <c r="F6" s="4" t="n">
         <v>275</v>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="J6" s="4" t="n">
         <v>260</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="K6" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="L6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="M6" s="4" t="n">
         <v>276</v>
       </c>
-      <c r="M6" s="4" t="n">
+      <c r="N6" s="4" t="n">
         <v>275</v>
       </c>
+      <c r="O6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1199,31 +1279,37 @@
       <c r="F7" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="J7" s="4" t="n">
         <v>240</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="K7" s="4" t="n">
         <v>130</v>
       </c>
-      <c r="K7" s="4" t="n">
+      <c r="L7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="L7" s="4" t="n">
+      <c r="M7" s="4" t="n">
         <v>287</v>
       </c>
-      <c r="M7" s="4" t="n">
+      <c r="N7" s="4" t="n">
         <v>280</v>
       </c>
+      <c r="O7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1248,31 +1334,37 @@
       <c r="F8" s="4" t="n">
         <v>312</v>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="J8" s="4" t="n">
         <v>270</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="K8" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="L8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="M8" s="4" t="n">
         <v>310</v>
       </c>
-      <c r="M8" s="4" t="n">
+      <c r="N8" s="4" t="n">
         <v>312</v>
       </c>
+      <c r="O8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1301,57 +1393,122 @@
       <c r="F9" s="4" t="n">
         <v>579</v>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="4" t="n">
+        <v>574</v>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>N/A (no specification)</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>N/A (no specification)</t>
         </is>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="J9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="L9" s="4" t="n">
+      <c r="M9" s="4" t="n">
         <v>573</v>
       </c>
-      <c r="M9" s="4" t="n">
+      <c r="N9" s="4" t="n">
         <v>579</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="O9" s="4" t="n">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>DO9</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio K</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>288</v>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>N/A (sin lote)</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>N/A (sin lote)</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="M10" s="4" t="n"/>
+      <c r="N10" s="4" t="n"/>
+      <c r="O10" s="4" t="n">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Rango de aceptación shown as a shaded band. DO8 has no specification; only lote markers are displayed. X-axis shows product and belonging Laboratorio.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Units: mOsm/kg. Markers: Lote 1 (orange), Lote 2 (green).</t>
+          <t>Rango de aceptación shown as a shaded band. Asterisk (*) markers: DO8 = 574, DO9 = 288. X-axis shows product and belonging Laboratorio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Units: mOsm/kg. Markers: Lote 1 (orange), Lote 2 (green), * (black star).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A14:I14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1380,7 +1537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eje X: Producto (DO1–DO8) + Laboratorio | Eje Y: Osmolalidad (mOsm/kg), paso 25 | Sombra: Rango de aceptación | Círculos: Lote 1 &amp; Lote 2</t>
+          <t>Eje X: Producto (DO1–DO9) + Laboratorio | Eje Y: Osmolalidad (mOsm/kg), paso 25 | Sombra: Rango de aceptación | Círculos: Lote 1 &amp; Lote 2 | *: valores adicionales</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync DO chart sheet note with theoretical value legend
Co-authored-by: Smansilla98 <Smansilla98@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/osmolality_results/osmolality_results.xlsx
+++ b/osmolality_results/osmolality_results.xlsx
@@ -359,7 +359,7 @@
           <idx val="4"/>
           <order val="4"/>
           <tx>
-            <v>*</v>
+            <v>Valor teórico estimado</v>
           </tx>
           <spPr>
             <a:ln>
@@ -1501,7 +1501,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Units: mOsm/kg. Markers: Lote 1 (orange), Lote 2 (green), * (black star).</t>
+          <t>Units: mOsm/kg. Markers: Lote 1 (orange), Lote 2 (green), estrella = Valor teórico estimado.</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eje X: Producto (DO1–DO9) + Laboratorio | Eje Y: Osmolalidad (mOsm/kg), paso 25 | Sombra: Rango de aceptación | Círculos: Lote 1 &amp; Lote 2 | *: valores adicionales</t>
+          <t>Eje X: Producto (DO1–DO9) + Laboratorio | Eje Y: Osmolalidad (mOsm/kg), paso 25 | Sombra: Rango de aceptación | Círculos: Lote 1 &amp; Lote 2 | Estrella: Valor teórico estimado</t>
         </is>
       </c>
     </row>

</xml_diff>